<commit_message>
Add 30 extended process routes and update Item Costing yield hints
Processes sheet now contains 47 routes covering CNC turning/milling,
welding variants, sheet-metal, casting, forging, heat treatment,
surface finishing, NDT and testing operations. YIELD_HINTS in
32_Item_Costing.py extended to match all new process IDs with
sensible material-utilisation defaults.

https://claude.ai/code/session_016MhJzUMJ3DpmWVaktTLWcD
</commit_message>
<xml_diff>
--- a/data/cost_forge.xlsx
+++ b/data/cost_forge.xlsx
@@ -533,7 +533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>3</v>
       </c>
@@ -584,7 +583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>2</v>
       </c>
@@ -635,7 +633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>2</v>
       </c>
@@ -686,7 +683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
         <v>2</v>
       </c>
@@ -737,7 +733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
         <v>2</v>
       </c>
@@ -788,7 +783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
         <v>1</v>
       </c>
@@ -839,7 +833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
         <v>2</v>
       </c>
@@ -890,7 +883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
         <v>1</v>
       </c>
@@ -941,7 +933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>0</v>
       </c>
@@ -992,7 +983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>0</v>
       </c>
@@ -1043,7 +1033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>0</v>
       </c>
@@ -1094,7 +1083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>0</v>
       </c>
@@ -1145,7 +1133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>3</v>
       </c>
@@ -1196,7 +1183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
         <v>2</v>
       </c>
@@ -1247,7 +1233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
         <v>2</v>
       </c>
@@ -1298,7 +1283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
         <v>2</v>
       </c>
@@ -1349,7 +1333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>2</v>
       </c>
@@ -1400,7 +1383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>1</v>
       </c>
@@ -1451,7 +1433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>0</v>
       </c>
@@ -1502,7 +1483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
         <v>2</v>
       </c>
@@ -1553,7 +1533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
         <v>0</v>
       </c>
@@ -1604,7 +1583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>0</v>
       </c>
@@ -1655,7 +1633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
         <v>3</v>
       </c>
@@ -1706,7 +1683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
         <v>3</v>
       </c>
@@ -1757,7 +1733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
         <v>2</v>
       </c>
@@ -1808,7 +1783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
         <v>0</v>
       </c>
@@ -1859,7 +1833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
         <v>2</v>
       </c>
@@ -1910,7 +1883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
         <v>2</v>
       </c>
@@ -1961,7 +1933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
         <v>2</v>
       </c>
@@ -2012,7 +1983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
         <v>2</v>
       </c>
@@ -2063,7 +2033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
         <v>1</v>
       </c>
@@ -2114,7 +2083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
         <v>1</v>
       </c>
@@ -2165,7 +2133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="n">
         <v>0</v>
       </c>
@@ -2216,7 +2183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
         <v>0</v>
       </c>
@@ -2267,7 +2233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
         <v>0</v>
       </c>
@@ -2318,7 +2283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" t="n">
         <v>2</v>
       </c>
@@ -2369,7 +2333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
         <v>0</v>
       </c>
@@ -2420,7 +2383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
         <v>2</v>
       </c>
@@ -2471,7 +2433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>2</v>
       </c>
@@ -2522,7 +2483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="n">
         <v>2</v>
       </c>
@@ -2573,7 +2533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
         <v>2</v>
       </c>
@@ -2624,7 +2583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
         <v>2</v>
       </c>
@@ -2675,7 +2633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>2</v>
       </c>
@@ -2726,7 +2683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
         <v>1</v>
       </c>
@@ -2777,7 +2733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
         <v>0</v>
       </c>
@@ -2828,7 +2783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
         <v>1</v>
       </c>
@@ -2879,7 +2833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
         <v>0</v>
       </c>
@@ -2930,7 +2883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="n">
         <v>0</v>
       </c>
@@ -2981,7 +2933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
         <v>0</v>
       </c>
@@ -3032,7 +2983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
         <v>2</v>
       </c>
@@ -3083,7 +3033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
         <v>2</v>
       </c>
@@ -3134,7 +3083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
       <c r="M53" t="n">
         <v>2</v>
       </c>
@@ -3185,7 +3133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" t="n">
         <v>0</v>
       </c>
@@ -3236,7 +3183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" t="n">
         <v>1</v>
       </c>
@@ -3287,7 +3233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="n">
         <v>2</v>
       </c>
@@ -3338,7 +3283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="n">
         <v>1</v>
       </c>
@@ -3389,7 +3333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="n">
         <v>0</v>
       </c>
@@ -3440,7 +3383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
         <v>0</v>
       </c>
@@ -3491,7 +3433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" t="n">
         <v>0</v>
       </c>
@@ -3542,7 +3483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
         <v>2</v>
       </c>
@@ -3593,7 +3533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
         <v>2</v>
       </c>
@@ -3644,7 +3583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>2</v>
       </c>
@@ -3695,7 +3633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr"/>
       <c r="M64" t="n">
         <v>2</v>
       </c>
@@ -3746,7 +3683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
         <v>2</v>
       </c>
@@ -3797,7 +3733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
       <c r="M66" t="n">
         <v>2</v>
       </c>
@@ -3848,7 +3783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
       <c r="M67" t="n">
         <v>2</v>
       </c>
@@ -3899,7 +3833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr"/>
       <c r="M68" t="n">
         <v>1</v>
       </c>
@@ -3950,7 +3883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr"/>
       <c r="M69" t="n">
         <v>0</v>
       </c>
@@ -4001,7 +3933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
       <c r="M70" t="n">
         <v>0</v>
       </c>
@@ -4052,7 +3983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="n">
         <v>0</v>
       </c>
@@ -4103,7 +4033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr"/>
       <c r="M72" t="n">
         <v>2</v>
       </c>
@@ -4154,7 +4083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" t="n">
         <v>2</v>
       </c>
@@ -4205,7 +4133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="n">
         <v>2</v>
       </c>
@@ -4256,7 +4183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" t="n">
         <v>2</v>
       </c>
@@ -4307,7 +4233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
       <c r="M76" t="n">
         <v>1</v>
       </c>
@@ -4358,7 +4283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="n">
         <v>1</v>
       </c>
@@ -4409,7 +4333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="n">
         <v>0</v>
       </c>
@@ -4460,7 +4383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" t="n">
         <v>0</v>
       </c>
@@ -4511,7 +4433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" t="n">
         <v>0</v>
       </c>
@@ -4562,7 +4483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
       <c r="M81" t="n">
         <v>2</v>
       </c>
@@ -4613,7 +4533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" t="n">
         <v>2</v>
       </c>
@@ -4664,7 +4583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr"/>
       <c r="M83" t="n">
         <v>2</v>
       </c>
@@ -4715,7 +4633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
       <c r="M84" t="n">
         <v>2</v>
       </c>
@@ -4766,7 +4683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr"/>
       <c r="M85" t="n">
         <v>2</v>
       </c>
@@ -4817,7 +4733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" t="n">
         <v>2</v>
       </c>
@@ -4868,7 +4783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" t="n">
         <v>1</v>
       </c>
@@ -4919,7 +4833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr"/>
       <c r="M88" t="n">
         <v>1</v>
       </c>
@@ -4970,7 +4883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr"/>
       <c r="M89" t="n">
         <v>1</v>
       </c>
@@ -5021,7 +4933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="n">
         <v>0</v>
       </c>
@@ -5072,7 +4983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="n">
         <v>2</v>
       </c>
@@ -5123,7 +5033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L92" t="inlineStr"/>
       <c r="M92" t="n">
         <v>2</v>
       </c>
@@ -5174,7 +5083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="n">
         <v>1</v>
       </c>
@@ -5225,7 +5133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>2</v>
       </c>
@@ -5276,7 +5183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
       <c r="M95" t="n">
         <v>2</v>
       </c>
@@ -5327,7 +5233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
       <c r="M96" t="n">
         <v>1</v>
       </c>
@@ -5378,7 +5283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="n">
         <v>1</v>
       </c>
@@ -5429,7 +5333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr"/>
       <c r="M98" t="n">
         <v>1</v>
       </c>
@@ -5480,7 +5383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr"/>
       <c r="M99" t="n">
         <v>0</v>
       </c>
@@ -5531,7 +5433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
       <c r="M100" t="n">
         <v>0</v>
       </c>
@@ -5582,7 +5483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
       <c r="M101" t="n">
         <v>2</v>
       </c>
@@ -5633,7 +5533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr"/>
       <c r="M102" t="n">
         <v>2</v>
       </c>
@@ -5684,7 +5583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr"/>
       <c r="M103" t="n">
         <v>2</v>
       </c>
@@ -5735,7 +5633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L104" t="inlineStr"/>
       <c r="M104" t="n">
         <v>2</v>
       </c>
@@ -5786,7 +5683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="n">
         <v>2</v>
       </c>
@@ -5837,7 +5733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>2</v>
       </c>
@@ -5888,7 +5783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L107" t="inlineStr"/>
       <c r="M107" t="n">
         <v>0</v>
       </c>
@@ -5939,7 +5833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L108" t="inlineStr"/>
       <c r="M108" t="n">
         <v>2</v>
       </c>
@@ -5990,7 +5883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L109" t="inlineStr"/>
       <c r="M109" t="n">
         <v>0</v>
       </c>
@@ -6041,7 +5933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>2</v>
       </c>
@@ -6092,7 +5983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L111" t="inlineStr"/>
       <c r="M111" t="n">
         <v>2</v>
       </c>
@@ -6143,7 +6033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr"/>
       <c r="M112" t="n">
         <v>0</v>
       </c>
@@ -6194,7 +6083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L113" t="inlineStr"/>
       <c r="M113" t="n">
         <v>1</v>
       </c>
@@ -6245,7 +6133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr"/>
       <c r="M114" t="n">
         <v>1</v>
       </c>
@@ -6296,7 +6183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L115" t="inlineStr"/>
       <c r="M115" t="n">
         <v>1</v>
       </c>
@@ -6347,7 +6233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L116" t="inlineStr"/>
       <c r="M116" t="n">
         <v>1</v>
       </c>
@@ -6398,7 +6283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L117" t="inlineStr"/>
       <c r="M117" t="n">
         <v>2</v>
       </c>
@@ -6449,7 +6333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L118" t="inlineStr"/>
       <c r="M118" t="n">
         <v>0</v>
       </c>
@@ -6500,7 +6383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L119" t="inlineStr"/>
       <c r="M119" t="n">
         <v>0</v>
       </c>
@@ -6551,7 +6433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L120" t="inlineStr"/>
       <c r="M120" t="n">
         <v>1</v>
       </c>
@@ -6602,7 +6483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L121" t="inlineStr"/>
       <c r="M121" t="n">
         <v>1</v>
       </c>
@@ -6653,7 +6533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L122" t="inlineStr"/>
       <c r="M122" t="n">
         <v>1</v>
       </c>
@@ -6704,7 +6583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L123" t="inlineStr"/>
       <c r="M123" t="n">
         <v>1</v>
       </c>
@@ -6755,7 +6633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr"/>
       <c r="M124" t="n">
         <v>1</v>
       </c>
@@ -6806,7 +6683,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr"/>
       <c r="M125" t="n">
         <v>1</v>
       </c>
@@ -6857,7 +6733,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr"/>
       <c r="M126" t="n">
         <v>1</v>
       </c>
@@ -6908,7 +6783,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr"/>
       <c r="M127" t="n">
         <v>0</v>
       </c>
@@ -6959,7 +6833,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr"/>
       <c r="M128" t="n">
         <v>0</v>
       </c>
@@ -7010,7 +6883,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr"/>
       <c r="M129" t="n">
         <v>0</v>
       </c>
@@ -7061,7 +6933,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr"/>
       <c r="M130" t="n">
         <v>0</v>
       </c>
@@ -7112,7 +6983,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr"/>
       <c r="M131" t="n">
         <v>0</v>
       </c>
@@ -7163,7 +7033,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr"/>
       <c r="M132" t="n">
         <v>0</v>
       </c>
@@ -7214,7 +7083,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr"/>
       <c r="M133" t="n">
         <v>0</v>
       </c>
@@ -7265,7 +7133,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr"/>
       <c r="M134" t="n">
         <v>0</v>
       </c>
@@ -7316,7 +7183,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr"/>
       <c r="M135" t="n">
         <v>0</v>
       </c>
@@ -7367,7 +7233,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr"/>
       <c r="M136" t="n">
         <v>0</v>
       </c>
@@ -7418,7 +7283,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr"/>
       <c r="M137" t="n">
         <v>0</v>
       </c>
@@ -7469,7 +7333,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L138" t="inlineStr"/>
       <c r="M138" t="n">
         <v>0</v>
       </c>
@@ -7520,7 +7383,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr"/>
       <c r="M139" t="n">
         <v>0</v>
       </c>
@@ -7571,7 +7433,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr"/>
       <c r="M140" t="n">
         <v>0</v>
       </c>
@@ -7622,7 +7483,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr"/>
       <c r="M141" t="n">
         <v>0</v>
       </c>
@@ -7673,7 +7533,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L142" t="inlineStr"/>
       <c r="M142" t="n">
         <v>0</v>
       </c>
@@ -7724,7 +7583,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L143" t="inlineStr"/>
       <c r="M143" t="n">
         <v>0</v>
       </c>
@@ -7775,7 +7633,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="L144" t="inlineStr"/>
       <c r="M144" t="n">
         <v>0</v>
       </c>
@@ -8147,7 +8004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8587,6 +8444,726 @@
         <v>0.2</v>
       </c>
       <c r="F18" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CNC_LATHE_GEN</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CNC turning — general purpose</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>65</v>
+      </c>
+      <c r="D19" t="n">
+        <v>45</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CNC_MILL_4AX</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4-axis CNC milling</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>120</v>
+      </c>
+      <c r="D20" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TURN_MILL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Turn-mill combined (multi-tasking centre)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>145</v>
+      </c>
+      <c r="D21" t="n">
+        <v>65</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DEEP_HOLE_DRILL</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Deep hole / gun drilling</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>95</v>
+      </c>
+      <c r="D22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HONING</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Internal honing (cylinders / bores)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>75</v>
+      </c>
+      <c r="D23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LAPPING</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Precision lapping (sealing faces)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>65</v>
+      </c>
+      <c r="D24" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>JIG_BORE</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jig boring — precision hole patterns</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" t="n">
+        <v>55</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>THREAD_GRIND</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Thread grinding (precision screws / nuts)</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>85</v>
+      </c>
+      <c r="D26" t="n">
+        <v>50</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GEAR_CUT</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gear cutting / hobbing</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>110</v>
+      </c>
+      <c r="D27" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MIG_WELD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MIG / MAG welding — structural</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>50</v>
+      </c>
+      <c r="D28" t="n">
+        <v>55</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PIPE_WELD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Pipe &amp; tube welding — certified</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>65</v>
+      </c>
+      <c r="D29" t="n">
+        <v>70</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>WELD_OVERLAY</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Weld overlay / hard-facing cladding</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>70</v>
+      </c>
+      <c r="D30" t="n">
+        <v>65</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LASER_WELD</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Laser welding — thin section precision</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>120</v>
+      </c>
+      <c r="D31" t="n">
+        <v>55</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LASER_CUT</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Laser cutting — sheet and plate</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>85</v>
+      </c>
+      <c r="D32" t="n">
+        <v>35</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FLAME_CUT</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Oxy-fuel cutting — heavy plate</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>55</v>
+      </c>
+      <c r="D33" t="n">
+        <v>35</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PRESS_BRAKE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Press brake forming — sheet / plate</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>60</v>
+      </c>
+      <c r="D34" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ROLL_FORM</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Plate / section rolling (cylinders, rings)</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>55</v>
+      </c>
+      <c r="D35" t="n">
+        <v>40</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>INVEST_CAST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Investment casting (lost-wax)</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>55</v>
+      </c>
+      <c r="D36" t="n">
+        <v>45</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CENTRIFUGAL</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Centrifugal casting (tubes / rings)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>50</v>
+      </c>
+      <c r="D37" t="n">
+        <v>40</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FORGING</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Drop forging — hot / warm</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>95</v>
+      </c>
+      <c r="D38" t="n">
+        <v>45</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>HEAT_TREAT</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Heat treatment (stress relief / anneal / quench)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>40</v>
+      </c>
+      <c r="D39" t="n">
+        <v>30</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SHOT_PEEN</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Shot peening (fatigue improvement)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>45</v>
+      </c>
+      <c r="D40" t="n">
+        <v>35</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HOT_DIP_GALV</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Hot-dip galvanising</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>40</v>
+      </c>
+      <c r="D41" t="n">
+        <v>30</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NITRIDING</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Gas / plasma nitriding</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>60</v>
+      </c>
+      <c r="D42" t="n">
+        <v>40</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RUBBER_BOND</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Rubber bonding / vulcanising</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>45</v>
+      </c>
+      <c r="D43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CMM_INSPECT</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CMM dimensional inspection</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>75</v>
+      </c>
+      <c r="D44" t="n">
+        <v>65</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RADIOGRAPHY</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>X-ray radiography NDT</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>90</v>
+      </c>
+      <c r="D45" t="n">
+        <v>75</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>FLOW_TEST</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Flow / performance acceptance test</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>60</v>
+      </c>
+      <c r="D46" t="n">
+        <v>55</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LEAK_TEST</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Helium / pneumatic leak test</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>55</v>
+      </c>
+      <c r="D47" t="n">
+        <v>50</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>VIBRATION_TEST</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Vibration / fatigue testing</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>70</v>
+      </c>
+      <c r="D48" t="n">
+        <v>60</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F48" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -9104,10 +9681,6 @@
           <t>I01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9120,10 +9693,6 @@
           <t>I02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9136,10 +9705,6 @@
           <t>I03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9152,10 +9717,6 @@
           <t>I04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9168,10 +9729,6 @@
           <t>I05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9184,10 +9741,6 @@
           <t>I06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9200,10 +9753,6 @@
           <t>I07</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9216,10 +9765,6 @@
           <t>I08</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9232,10 +9777,6 @@
           <t>I09</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9248,10 +9789,6 @@
           <t>I10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9264,10 +9801,6 @@
           <t>I11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9280,10 +9813,6 @@
           <t>I12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9296,10 +9825,6 @@
           <t>SB01</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9312,10 +9837,6 @@
           <t>SB02</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9328,10 +9849,6 @@
           <t>SB03</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9344,10 +9861,6 @@
           <t>SB04</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9360,10 +9873,6 @@
           <t>SB05</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9376,10 +9885,6 @@
           <t>SB06</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9392,10 +9897,6 @@
           <t>SB07</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9408,10 +9909,6 @@
           <t>SB08</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9424,10 +9921,6 @@
           <t>SB09</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9440,10 +9933,6 @@
           <t>SB10</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9456,10 +9945,6 @@
           <t>H01</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9472,10 +9957,6 @@
           <t>H02</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9488,10 +9969,6 @@
           <t>H03</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9504,10 +9981,6 @@
           <t>H04</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9520,10 +9993,6 @@
           <t>H05</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9536,10 +10005,6 @@
           <t>H06</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9552,10 +10017,6 @@
           <t>H07</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9568,10 +10029,6 @@
           <t>H08</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9584,10 +10041,6 @@
           <t>H09</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9600,10 +10053,6 @@
           <t>H10</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9616,10 +10065,6 @@
           <t>H11</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9632,10 +10077,6 @@
           <t>H12</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9648,10 +10089,6 @@
           <t>H13</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9664,10 +10101,6 @@
           <t>S01</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9680,10 +10113,6 @@
           <t>S02</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9696,10 +10125,6 @@
           <t>S03</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9712,10 +10137,6 @@
           <t>S04</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9728,10 +10149,6 @@
           <t>S05</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9744,10 +10161,6 @@
           <t>S06</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9760,10 +10173,6 @@
           <t>S07</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9776,10 +10185,6 @@
           <t>S08</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9792,10 +10197,6 @@
           <t>S09</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9808,10 +10209,6 @@
           <t>S10</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9824,10 +10221,6 @@
           <t>S11</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9840,10 +10233,6 @@
           <t>S12</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9856,10 +10245,6 @@
           <t>S13</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9872,10 +10257,6 @@
           <t>S14</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9888,10 +10269,6 @@
           <t>TB01</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9904,10 +10281,6 @@
           <t>TB02</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9920,10 +10293,6 @@
           <t>TB03</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9936,10 +10305,6 @@
           <t>TB04</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9952,10 +10317,6 @@
           <t>TB05</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9968,10 +10329,6 @@
           <t>TB06</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -9984,10 +10341,6 @@
           <t>TB07</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10000,10 +10353,6 @@
           <t>TB08</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10016,10 +10365,6 @@
           <t>TB09</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10032,10 +10377,6 @@
           <t>TB10</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10048,10 +10389,6 @@
           <t>D01</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10064,10 +10401,6 @@
           <t>D02</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10080,10 +10413,6 @@
           <t>D03</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10096,10 +10425,6 @@
           <t>D04</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10112,10 +10437,6 @@
           <t>D05</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10128,10 +10449,6 @@
           <t>D06</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10144,10 +10461,6 @@
           <t>D07</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10160,10 +10473,6 @@
           <t>D08</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10176,10 +10485,6 @@
           <t>D09</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10192,10 +10497,6 @@
           <t>D10</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10208,10 +10509,6 @@
           <t>D11</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10224,10 +10521,6 @@
           <t>N01</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10240,10 +10533,6 @@
           <t>N02</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10256,10 +10545,6 @@
           <t>N03</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10272,10 +10557,6 @@
           <t>N04</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10288,10 +10569,6 @@
           <t>N05</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10304,10 +10581,6 @@
           <t>N06</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10320,10 +10593,6 @@
           <t>N07</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10336,10 +10605,6 @@
           <t>N08</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10352,10 +10617,6 @@
           <t>N09</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10368,10 +10629,6 @@
           <t>ST01</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10384,10 +10641,6 @@
           <t>ST02</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10400,10 +10653,6 @@
           <t>ST03</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10416,10 +10665,6 @@
           <t>ST04</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10432,10 +10677,6 @@
           <t>ST05</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10448,10 +10689,6 @@
           <t>ST06</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10464,10 +10701,6 @@
           <t>ST07</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10480,10 +10713,6 @@
           <t>ST08</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10496,10 +10725,6 @@
           <t>ST09</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10512,10 +10737,6 @@
           <t>ST10</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10528,10 +10749,6 @@
           <t>R01</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10544,10 +10761,6 @@
           <t>R02</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10560,10 +10773,6 @@
           <t>R03</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10576,10 +10785,6 @@
           <t>R04</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10592,10 +10797,6 @@
           <t>R05</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10608,10 +10809,6 @@
           <t>R06</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10624,10 +10821,6 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10640,10 +10833,6 @@
           <t>R08</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10656,10 +10845,6 @@
           <t>R09</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10672,10 +10857,6 @@
           <t>R10</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10688,10 +10869,6 @@
           <t>F01</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10704,10 +10881,6 @@
           <t>F02</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10720,10 +10893,6 @@
           <t>F03</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10736,10 +10905,6 @@
           <t>F04</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10752,10 +10917,6 @@
           <t>F05</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10768,10 +10929,6 @@
           <t>F06</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10784,10 +10941,6 @@
           <t>F07</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10800,10 +10953,6 @@
           <t>F08</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10816,10 +10965,6 @@
           <t>F09</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10832,10 +10977,6 @@
           <t>SE01</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10848,10 +10989,6 @@
           <t>SE02</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10864,10 +11001,6 @@
           <t>SE03</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10880,10 +11013,6 @@
           <t>SE04</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10896,10 +11025,6 @@
           <t>SE05</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
-      <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10912,10 +11037,6 @@
           <t>SE06</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10928,10 +11049,6 @@
           <t>SE07</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10944,10 +11061,6 @@
           <t>SE08</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10960,10 +11073,6 @@
           <t>SE09</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10976,10 +11085,6 @@
           <t>SE10</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -10992,10 +11097,6 @@
           <t>HY01</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11008,10 +11109,6 @@
           <t>HY02</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11024,10 +11121,6 @@
           <t>HY03</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11040,10 +11133,6 @@
           <t>HY04</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11056,10 +11145,6 @@
           <t>HY05</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11072,10 +11157,6 @@
           <t>HY06</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11088,10 +11169,6 @@
           <t>HY07</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11104,10 +11181,6 @@
           <t>HY08</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11120,10 +11193,6 @@
           <t>HY09</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
-      <c r="C128" t="inlineStr"/>
-      <c r="D128" t="inlineStr"/>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11136,10 +11205,6 @@
           <t>HW01</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
-      <c r="D129" t="inlineStr"/>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11152,10 +11217,6 @@
           <t>HW02</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
-      <c r="D130" t="inlineStr"/>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11168,10 +11229,6 @@
           <t>HW03</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
-      <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11184,10 +11241,6 @@
           <t>HW04</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
-      <c r="C132" t="inlineStr"/>
-      <c r="D132" t="inlineStr"/>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11200,10 +11253,6 @@
           <t>HW05</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
-      <c r="C133" t="inlineStr"/>
-      <c r="D133" t="inlineStr"/>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11216,10 +11265,6 @@
           <t>HW06</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
-      <c r="C134" t="inlineStr"/>
-      <c r="D134" t="inlineStr"/>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11232,10 +11277,6 @@
           <t>HW07</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11248,10 +11289,6 @@
           <t>HW08</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11264,10 +11301,6 @@
           <t>QA01</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11280,10 +11313,6 @@
           <t>QA02</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11296,10 +11325,6 @@
           <t>QA03</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11312,10 +11337,6 @@
           <t>QA04</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr"/>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11328,10 +11349,6 @@
           <t>QA05</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11344,10 +11361,6 @@
           <t>QA06</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11360,10 +11373,6 @@
           <t>QA07</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>not_started</t>
@@ -11376,10 +11385,6 @@
           <t>QA08</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>not_started</t>

</xml_diff>